<commit_message>
Promote 10 readiness-stage cases to TIER2_PASS/published; update roadmap
Re-verified airplane-manufacturer, airstrike, wildfire, redrawing-lines,
and family-trip against the live gate scripts rather than trusting
self-reported case.json state — found and fixed real defects along the
way (a facilitator-content leak in build_docx.js's HTML-comment strip,
a qa.verdict schema typo, two bad P6 citations on family-trip, a missing
published/ packet on redrawing-lines) before promoting each to published.
Also caught and repaired a promotion-script regression that had silently
stripped coverage credit from two cases' covered_by[] during a later
promotion. ROADMAP.md gets a new v2.10 entry documenting the chunk-of-10
results and the current major skill-gap picture (73 uncovered skills,
19 groups) against the already-scoped next-10-careers concept queue.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cases/cold-chain/published/Cold Chain - Student Workbook.xlsx
+++ b/cases/cold-chain/published/Cold Chain - Student Workbook.xlsx
@@ -665,7 +665,7 @@
         <v>25.4</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>102.21</v>
+        <v>76.78</v>
       </c>
     </row>
     <row r="8">
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>102.21</v>
+        <v>76.78</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>128</v>

</xml_diff>